<commit_message>
Stabilisation saisie P1 - DV M04 IK
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/02_DONNEES_NORMALISEES/menages/M04_MENAGES_PowerQuery.xlsx
+++ b/02_DONNEES_NORMALISEES/menages/M04_MENAGES_PowerQuery.xlsx
@@ -563,7 +563,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
@@ -625,15 +625,20 @@
       </c>
     </row>
   </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="C2:C501" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Valeur hors liste" error="Valeur non listee. Verifier l'orthographe ou completer le referentiel." promptTitle="Liste" prompt="Intervenant (PARAM_TAUX_INTERVENANTS)" type="list" errorStyle="warning">
+      <formula1>=PARAM_TAUX_INTERVENANTS!$B$2:$B$6</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </tableParts>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
@@ -862,13 +867,13 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </tableParts>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
@@ -946,7 +951,7 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Pipeline menages - runner ordre garanti lot6b avant 6d/6e/6f
</commit_message>
<xml_diff>
--- a/02_DONNEES_NORMALISEES/menages/M04_MENAGES_PowerQuery.xlsx
+++ b/02_DONNEES_NORMALISEES/menages/M04_MENAGES_PowerQuery.xlsx
@@ -1963,7 +1963,7 @@
       </c>
       <c r="AH2" t="inlineStr">
         <is>
-          <t>2026-06-18T11:22:24</t>
+          <t>2026-06-18T11:33:09</t>
         </is>
       </c>
     </row>
@@ -2110,7 +2110,7 @@
       </c>
       <c r="AH3" t="inlineStr">
         <is>
-          <t>2026-06-18T11:22:24</t>
+          <t>2026-06-18T11:33:09</t>
         </is>
       </c>
     </row>
@@ -2257,7 +2257,7 @@
       </c>
       <c r="AH4" t="inlineStr">
         <is>
-          <t>2026-06-18T11:22:24</t>
+          <t>2026-06-18T11:33:09</t>
         </is>
       </c>
     </row>
@@ -2404,7 +2404,7 @@
       </c>
       <c r="AH5" t="inlineStr">
         <is>
-          <t>2026-06-18T11:22:24</t>
+          <t>2026-06-18T11:33:09</t>
         </is>
       </c>
     </row>
@@ -2551,7 +2551,7 @@
       </c>
       <c r="AH6" t="inlineStr">
         <is>
-          <t>2026-06-18T11:22:24</t>
+          <t>2026-06-18T11:33:09</t>
         </is>
       </c>
     </row>
@@ -2698,7 +2698,7 @@
       </c>
       <c r="AH7" t="inlineStr">
         <is>
-          <t>2026-06-18T11:22:24</t>
+          <t>2026-06-18T11:33:09</t>
         </is>
       </c>
     </row>
@@ -2845,7 +2845,7 @@
       </c>
       <c r="AH8" t="inlineStr">
         <is>
-          <t>2026-06-18T11:22:24</t>
+          <t>2026-06-18T11:33:09</t>
         </is>
       </c>
     </row>
@@ -2992,7 +2992,7 @@
       </c>
       <c r="AH9" t="inlineStr">
         <is>
-          <t>2026-06-18T11:22:24</t>
+          <t>2026-06-18T11:33:09</t>
         </is>
       </c>
     </row>
@@ -3139,7 +3139,7 @@
       </c>
       <c r="AH10" t="inlineStr">
         <is>
-          <t>2026-06-18T11:22:24</t>
+          <t>2026-06-18T11:33:09</t>
         </is>
       </c>
     </row>
@@ -3286,7 +3286,7 @@
       </c>
       <c r="AH11" t="inlineStr">
         <is>
-          <t>2026-06-18T11:22:24</t>
+          <t>2026-06-18T11:33:09</t>
         </is>
       </c>
     </row>
@@ -3433,7 +3433,7 @@
       </c>
       <c r="AH12" t="inlineStr">
         <is>
-          <t>2026-06-18T11:22:24</t>
+          <t>2026-06-18T11:33:09</t>
         </is>
       </c>
     </row>
@@ -3580,7 +3580,7 @@
       </c>
       <c r="AH13" t="inlineStr">
         <is>
-          <t>2026-06-18T11:22:24</t>
+          <t>2026-06-18T11:33:09</t>
         </is>
       </c>
     </row>
@@ -3727,7 +3727,7 @@
       </c>
       <c r="AH14" t="inlineStr">
         <is>
-          <t>2026-06-18T11:22:24</t>
+          <t>2026-06-18T11:33:09</t>
         </is>
       </c>
     </row>
@@ -3874,7 +3874,7 @@
       </c>
       <c r="AH15" t="inlineStr">
         <is>
-          <t>2026-06-18T11:22:24</t>
+          <t>2026-06-18T11:33:09</t>
         </is>
       </c>
     </row>
@@ -4021,7 +4021,7 @@
       </c>
       <c r="AH16" t="inlineStr">
         <is>
-          <t>2026-06-18T11:22:24</t>
+          <t>2026-06-18T11:33:09</t>
         </is>
       </c>
     </row>
@@ -4168,7 +4168,7 @@
       </c>
       <c r="AH17" t="inlineStr">
         <is>
-          <t>2026-06-18T11:22:24</t>
+          <t>2026-06-18T11:33:09</t>
         </is>
       </c>
     </row>
@@ -4315,7 +4315,7 @@
       </c>
       <c r="AH18" t="inlineStr">
         <is>
-          <t>2026-06-18T11:22:24</t>
+          <t>2026-06-18T11:33:09</t>
         </is>
       </c>
     </row>
@@ -4462,7 +4462,7 @@
       </c>
       <c r="AH19" t="inlineStr">
         <is>
-          <t>2026-06-18T11:22:24</t>
+          <t>2026-06-18T11:33:09</t>
         </is>
       </c>
     </row>
@@ -4594,7 +4594,7 @@
       </c>
       <c r="AH20" t="inlineStr">
         <is>
-          <t>2026-06-18T11:22:24</t>
+          <t>2026-06-18T11:33:09</t>
         </is>
       </c>
     </row>
@@ -4726,7 +4726,7 @@
       </c>
       <c r="AH21" t="inlineStr">
         <is>
-          <t>2026-06-18T11:22:24</t>
+          <t>2026-06-18T11:33:09</t>
         </is>
       </c>
     </row>
@@ -5095,7 +5095,7 @@
       </c>
       <c r="AH2" t="inlineStr">
         <is>
-          <t>2026-06-18T11:22:24</t>
+          <t>2026-06-18T11:33:09</t>
         </is>
       </c>
     </row>
@@ -5242,7 +5242,7 @@
       </c>
       <c r="AH3" t="inlineStr">
         <is>
-          <t>2026-06-18T11:22:24</t>
+          <t>2026-06-18T11:33:09</t>
         </is>
       </c>
     </row>
@@ -5389,7 +5389,7 @@
       </c>
       <c r="AH4" t="inlineStr">
         <is>
-          <t>2026-06-18T11:22:24</t>
+          <t>2026-06-18T11:33:09</t>
         </is>
       </c>
     </row>
@@ -5536,7 +5536,7 @@
       </c>
       <c r="AH5" t="inlineStr">
         <is>
-          <t>2026-06-18T11:22:24</t>
+          <t>2026-06-18T11:33:09</t>
         </is>
       </c>
     </row>
@@ -5683,7 +5683,7 @@
       </c>
       <c r="AH6" t="inlineStr">
         <is>
-          <t>2026-06-18T11:22:24</t>
+          <t>2026-06-18T11:33:09</t>
         </is>
       </c>
     </row>
@@ -5830,7 +5830,7 @@
       </c>
       <c r="AH7" t="inlineStr">
         <is>
-          <t>2026-06-18T11:22:24</t>
+          <t>2026-06-18T11:33:09</t>
         </is>
       </c>
     </row>
@@ -5977,7 +5977,7 @@
       </c>
       <c r="AH8" t="inlineStr">
         <is>
-          <t>2026-06-18T11:22:24</t>
+          <t>2026-06-18T11:33:09</t>
         </is>
       </c>
     </row>
@@ -6124,7 +6124,7 @@
       </c>
       <c r="AH9" t="inlineStr">
         <is>
-          <t>2026-06-18T11:22:24</t>
+          <t>2026-06-18T11:33:09</t>
         </is>
       </c>
     </row>
@@ -6271,7 +6271,7 @@
       </c>
       <c r="AH10" t="inlineStr">
         <is>
-          <t>2026-06-18T11:22:24</t>
+          <t>2026-06-18T11:33:09</t>
         </is>
       </c>
     </row>
@@ -6418,7 +6418,7 @@
       </c>
       <c r="AH11" t="inlineStr">
         <is>
-          <t>2026-06-18T11:22:24</t>
+          <t>2026-06-18T11:33:09</t>
         </is>
       </c>
     </row>
@@ -6565,7 +6565,7 @@
       </c>
       <c r="AH12" t="inlineStr">
         <is>
-          <t>2026-06-18T11:22:24</t>
+          <t>2026-06-18T11:33:09</t>
         </is>
       </c>
     </row>
@@ -6712,7 +6712,7 @@
       </c>
       <c r="AH13" t="inlineStr">
         <is>
-          <t>2026-06-18T11:22:24</t>
+          <t>2026-06-18T11:33:09</t>
         </is>
       </c>
     </row>
@@ -6859,7 +6859,7 @@
       </c>
       <c r="AH14" t="inlineStr">
         <is>
-          <t>2026-06-18T11:22:24</t>
+          <t>2026-06-18T11:33:09</t>
         </is>
       </c>
     </row>
@@ -7006,7 +7006,7 @@
       </c>
       <c r="AH15" t="inlineStr">
         <is>
-          <t>2026-06-18T11:22:24</t>
+          <t>2026-06-18T11:33:09</t>
         </is>
       </c>
     </row>
@@ -7153,7 +7153,7 @@
       </c>
       <c r="AH16" t="inlineStr">
         <is>
-          <t>2026-06-18T11:22:24</t>
+          <t>2026-06-18T11:33:09</t>
         </is>
       </c>
     </row>
@@ -7300,7 +7300,7 @@
       </c>
       <c r="AH17" t="inlineStr">
         <is>
-          <t>2026-06-18T11:22:24</t>
+          <t>2026-06-18T11:33:09</t>
         </is>
       </c>
     </row>
@@ -7447,7 +7447,7 @@
       </c>
       <c r="AH18" t="inlineStr">
         <is>
-          <t>2026-06-18T11:22:24</t>
+          <t>2026-06-18T11:33:09</t>
         </is>
       </c>
     </row>
@@ -7594,7 +7594,7 @@
       </c>
       <c r="AH19" t="inlineStr">
         <is>
-          <t>2026-06-18T11:22:24</t>
+          <t>2026-06-18T11:33:09</t>
         </is>
       </c>
     </row>
@@ -7726,7 +7726,7 @@
       </c>
       <c r="AH20" t="inlineStr">
         <is>
-          <t>2026-06-18T11:22:24</t>
+          <t>2026-06-18T11:33:09</t>
         </is>
       </c>
     </row>
@@ -7858,7 +7858,7 @@
       </c>
       <c r="AH21" t="inlineStr">
         <is>
-          <t>2026-06-18T11:22:24</t>
+          <t>2026-06-18T11:33:09</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Ecart analytique menage en HORS_COMPTA (TYPE_FLUX_018) - M04 013 analytique seul
</commit_message>
<xml_diff>
--- a/02_DONNEES_NORMALISEES/menages/M04_MENAGES_PowerQuery.xlsx
+++ b/02_DONNEES_NORMALISEES/menages/M04_MENAGES_PowerQuery.xlsx
@@ -1963,7 +1963,7 @@
       </c>
       <c r="AH2" t="inlineStr">
         <is>
-          <t>2026-06-18T11:33:09</t>
+          <t>2026-06-18T12:10:45</t>
         </is>
       </c>
     </row>
@@ -2110,7 +2110,7 @@
       </c>
       <c r="AH3" t="inlineStr">
         <is>
-          <t>2026-06-18T11:33:09</t>
+          <t>2026-06-18T12:10:45</t>
         </is>
       </c>
     </row>
@@ -2257,7 +2257,7 @@
       </c>
       <c r="AH4" t="inlineStr">
         <is>
-          <t>2026-06-18T11:33:09</t>
+          <t>2026-06-18T12:10:45</t>
         </is>
       </c>
     </row>
@@ -2404,7 +2404,7 @@
       </c>
       <c r="AH5" t="inlineStr">
         <is>
-          <t>2026-06-18T11:33:09</t>
+          <t>2026-06-18T12:10:45</t>
         </is>
       </c>
     </row>
@@ -2551,7 +2551,7 @@
       </c>
       <c r="AH6" t="inlineStr">
         <is>
-          <t>2026-06-18T11:33:09</t>
+          <t>2026-06-18T12:10:45</t>
         </is>
       </c>
     </row>
@@ -2698,7 +2698,7 @@
       </c>
       <c r="AH7" t="inlineStr">
         <is>
-          <t>2026-06-18T11:33:09</t>
+          <t>2026-06-18T12:10:45</t>
         </is>
       </c>
     </row>
@@ -2845,7 +2845,7 @@
       </c>
       <c r="AH8" t="inlineStr">
         <is>
-          <t>2026-06-18T11:33:09</t>
+          <t>2026-06-18T12:10:45</t>
         </is>
       </c>
     </row>
@@ -2992,7 +2992,7 @@
       </c>
       <c r="AH9" t="inlineStr">
         <is>
-          <t>2026-06-18T11:33:09</t>
+          <t>2026-06-18T12:10:45</t>
         </is>
       </c>
     </row>
@@ -3139,7 +3139,7 @@
       </c>
       <c r="AH10" t="inlineStr">
         <is>
-          <t>2026-06-18T11:33:09</t>
+          <t>2026-06-18T12:10:45</t>
         </is>
       </c>
     </row>
@@ -3286,7 +3286,7 @@
       </c>
       <c r="AH11" t="inlineStr">
         <is>
-          <t>2026-06-18T11:33:09</t>
+          <t>2026-06-18T12:10:45</t>
         </is>
       </c>
     </row>
@@ -3433,7 +3433,7 @@
       </c>
       <c r="AH12" t="inlineStr">
         <is>
-          <t>2026-06-18T11:33:09</t>
+          <t>2026-06-18T12:10:45</t>
         </is>
       </c>
     </row>
@@ -3580,7 +3580,7 @@
       </c>
       <c r="AH13" t="inlineStr">
         <is>
-          <t>2026-06-18T11:33:09</t>
+          <t>2026-06-18T12:10:45</t>
         </is>
       </c>
     </row>
@@ -3727,7 +3727,7 @@
       </c>
       <c r="AH14" t="inlineStr">
         <is>
-          <t>2026-06-18T11:33:09</t>
+          <t>2026-06-18T12:10:45</t>
         </is>
       </c>
     </row>
@@ -3874,7 +3874,7 @@
       </c>
       <c r="AH15" t="inlineStr">
         <is>
-          <t>2026-06-18T11:33:09</t>
+          <t>2026-06-18T12:10:45</t>
         </is>
       </c>
     </row>
@@ -4021,7 +4021,7 @@
       </c>
       <c r="AH16" t="inlineStr">
         <is>
-          <t>2026-06-18T11:33:09</t>
+          <t>2026-06-18T12:10:45</t>
         </is>
       </c>
     </row>
@@ -4168,7 +4168,7 @@
       </c>
       <c r="AH17" t="inlineStr">
         <is>
-          <t>2026-06-18T11:33:09</t>
+          <t>2026-06-18T12:10:45</t>
         </is>
       </c>
     </row>
@@ -4315,7 +4315,7 @@
       </c>
       <c r="AH18" t="inlineStr">
         <is>
-          <t>2026-06-18T11:33:09</t>
+          <t>2026-06-18T12:10:45</t>
         </is>
       </c>
     </row>
@@ -4462,7 +4462,7 @@
       </c>
       <c r="AH19" t="inlineStr">
         <is>
-          <t>2026-06-18T11:33:09</t>
+          <t>2026-06-18T12:10:45</t>
         </is>
       </c>
     </row>
@@ -4594,7 +4594,7 @@
       </c>
       <c r="AH20" t="inlineStr">
         <is>
-          <t>2026-06-18T11:33:09</t>
+          <t>2026-06-18T12:10:45</t>
         </is>
       </c>
     </row>
@@ -4726,7 +4726,7 @@
       </c>
       <c r="AH21" t="inlineStr">
         <is>
-          <t>2026-06-18T11:33:09</t>
+          <t>2026-06-18T12:10:45</t>
         </is>
       </c>
     </row>
@@ -5095,7 +5095,7 @@
       </c>
       <c r="AH2" t="inlineStr">
         <is>
-          <t>2026-06-18T11:33:09</t>
+          <t>2026-06-18T12:10:45</t>
         </is>
       </c>
     </row>
@@ -5242,7 +5242,7 @@
       </c>
       <c r="AH3" t="inlineStr">
         <is>
-          <t>2026-06-18T11:33:09</t>
+          <t>2026-06-18T12:10:45</t>
         </is>
       </c>
     </row>
@@ -5389,7 +5389,7 @@
       </c>
       <c r="AH4" t="inlineStr">
         <is>
-          <t>2026-06-18T11:33:09</t>
+          <t>2026-06-18T12:10:45</t>
         </is>
       </c>
     </row>
@@ -5536,7 +5536,7 @@
       </c>
       <c r="AH5" t="inlineStr">
         <is>
-          <t>2026-06-18T11:33:09</t>
+          <t>2026-06-18T12:10:45</t>
         </is>
       </c>
     </row>
@@ -5683,7 +5683,7 @@
       </c>
       <c r="AH6" t="inlineStr">
         <is>
-          <t>2026-06-18T11:33:09</t>
+          <t>2026-06-18T12:10:45</t>
         </is>
       </c>
     </row>
@@ -5830,7 +5830,7 @@
       </c>
       <c r="AH7" t="inlineStr">
         <is>
-          <t>2026-06-18T11:33:09</t>
+          <t>2026-06-18T12:10:45</t>
         </is>
       </c>
     </row>
@@ -5977,7 +5977,7 @@
       </c>
       <c r="AH8" t="inlineStr">
         <is>
-          <t>2026-06-18T11:33:09</t>
+          <t>2026-06-18T12:10:45</t>
         </is>
       </c>
     </row>
@@ -6124,7 +6124,7 @@
       </c>
       <c r="AH9" t="inlineStr">
         <is>
-          <t>2026-06-18T11:33:09</t>
+          <t>2026-06-18T12:10:45</t>
         </is>
       </c>
     </row>
@@ -6271,7 +6271,7 @@
       </c>
       <c r="AH10" t="inlineStr">
         <is>
-          <t>2026-06-18T11:33:09</t>
+          <t>2026-06-18T12:10:45</t>
         </is>
       </c>
     </row>
@@ -6418,7 +6418,7 @@
       </c>
       <c r="AH11" t="inlineStr">
         <is>
-          <t>2026-06-18T11:33:09</t>
+          <t>2026-06-18T12:10:45</t>
         </is>
       </c>
     </row>
@@ -6565,7 +6565,7 @@
       </c>
       <c r="AH12" t="inlineStr">
         <is>
-          <t>2026-06-18T11:33:09</t>
+          <t>2026-06-18T12:10:45</t>
         </is>
       </c>
     </row>
@@ -6712,7 +6712,7 @@
       </c>
       <c r="AH13" t="inlineStr">
         <is>
-          <t>2026-06-18T11:33:09</t>
+          <t>2026-06-18T12:10:45</t>
         </is>
       </c>
     </row>
@@ -6859,7 +6859,7 @@
       </c>
       <c r="AH14" t="inlineStr">
         <is>
-          <t>2026-06-18T11:33:09</t>
+          <t>2026-06-18T12:10:45</t>
         </is>
       </c>
     </row>
@@ -7006,7 +7006,7 @@
       </c>
       <c r="AH15" t="inlineStr">
         <is>
-          <t>2026-06-18T11:33:09</t>
+          <t>2026-06-18T12:10:45</t>
         </is>
       </c>
     </row>
@@ -7153,7 +7153,7 @@
       </c>
       <c r="AH16" t="inlineStr">
         <is>
-          <t>2026-06-18T11:33:09</t>
+          <t>2026-06-18T12:10:45</t>
         </is>
       </c>
     </row>
@@ -7300,7 +7300,7 @@
       </c>
       <c r="AH17" t="inlineStr">
         <is>
-          <t>2026-06-18T11:33:09</t>
+          <t>2026-06-18T12:10:45</t>
         </is>
       </c>
     </row>
@@ -7447,7 +7447,7 @@
       </c>
       <c r="AH18" t="inlineStr">
         <is>
-          <t>2026-06-18T11:33:09</t>
+          <t>2026-06-18T12:10:45</t>
         </is>
       </c>
     </row>
@@ -7594,7 +7594,7 @@
       </c>
       <c r="AH19" t="inlineStr">
         <is>
-          <t>2026-06-18T11:33:09</t>
+          <t>2026-06-18T12:10:45</t>
         </is>
       </c>
     </row>
@@ -7726,7 +7726,7 @@
       </c>
       <c r="AH20" t="inlineStr">
         <is>
-          <t>2026-06-18T11:33:09</t>
+          <t>2026-06-18T12:10:45</t>
         </is>
       </c>
     </row>
@@ -7858,7 +7858,7 @@
       </c>
       <c r="AH21" t="inlineStr">
         <is>
-          <t>2026-06-18T11:33:09</t>
+          <t>2026-06-18T12:10:45</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Audit fixes - README M04 et notes outils fictifs
</commit_message>
<xml_diff>
--- a/02_DONNEES_NORMALISEES/menages/M04_MENAGES_PowerQuery.xlsx
+++ b/02_DONNEES_NORMALISEES/menages/M04_MENAGES_PowerQuery.xlsx
@@ -8346,7 +8346,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B40"/>
+  <dimension ref="A1:B43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8583,9 +8583,10 @@
           <t>cout_execution_total</t>
         </is>
       </c>
-      <c r="B24" s="15">
-        <f> nb_heures × taux_horaire_intervenant</f>
-        <v/>
+      <c r="B24" s="15" t="inlineStr">
+        <is>
+          <t>'= nb_heures × taux_horaire_intervenant</t>
+        </is>
       </c>
     </row>
     <row r="25">
@@ -8594,9 +8595,10 @@
           <t>cout_standard_total_ligne</t>
         </is>
       </c>
-      <c r="B25" s="15">
-        <f> nb_menages × cout_standard  [BASE PONDÉRATION — non comptable]</f>
-        <v/>
+      <c r="B25" s="15" t="inlineStr">
+        <is>
+          <t>'= nb_menages × cout_standard  [BASE PONDÉRATION — non comptable]</t>
+        </is>
       </c>
     </row>
     <row r="26">
@@ -8605,9 +8607,10 @@
           <t>ecart_main_oeuvre_vs_standard</t>
         </is>
       </c>
-      <c r="B26" s="15">
-        <f> cout_standard − cout_execution_unitaire  (positif = favorable)</f>
-        <v/>
+      <c r="B26" s="15" t="inlineStr">
+        <is>
+          <t>'= cout_standard − cout_execution_unitaire  (positif = favorable)</t>
+        </is>
       </c>
     </row>
     <row r="27">
@@ -8739,6 +8742,20 @@
       <c r="B40" s="15" t="inlineStr">
         <is>
           <t>total_execution = cout_execution_total (colonne distincte, étape 10bis). Aucun doublon.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>NOTE (audit 2026-06-18)</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>M04 alimenté par script déterministe lot6b depuis Google Sheet (REF_Sources_Systeme SRC_011). 'PowerQuery' = nom historique, Power Query non utilisé.</t>
         </is>
       </c>
     </row>

</xml_diff>